<commit_message>
Update Word cloud - complete.xlsx
</commit_message>
<xml_diff>
--- a/Getting started/Word cloud - complete.xlsx
+++ b/Getting started/Word cloud - complete.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="49" documentId="8_{68B1EE44-EE51-4F8E-9F1B-857B7D4A1A03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB00D110-032B-47BB-83A3-CFF7ECB2376F}"/>
   <bookViews>
-    <workbookView xWindow="105" yWindow="-16320" windowWidth="29040" windowHeight="16440" xr2:uid="{36314F3C-7E5D-4645-BA3F-AC0B91DF8DC9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{36314F3C-7E5D-4645-BA3F-AC0B91DF8DC9}"/>
   </bookViews>
   <sheets>
     <sheet name="Wordcloud" sheetId="1" r:id="rId1"/>
@@ -691,12 +691,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="2"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="4"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -707,6 +701,12 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="5"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Heading 1" xfId="1" builtinId="16"/>
@@ -891,8 +891,8 @@
       <xdr:row>14</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer" Requires="sle15">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
+      <mc:Choice Requires="sle15">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="7" name="Gender">
@@ -915,7 +915,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -1722,22 +1722,22 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="4" t="e" vm="1">
+      <c r="B2" s="10" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="10"/>
     </row>
     <row r="4" spans="2:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="5"/>
+      <c r="C4" s="11"/>
       <c r="D4" s="2"/>
     </row>
     <row r="5" spans="2:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
@@ -1767,7 +1767,7 @@
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="9" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2068,15 +2068,15 @@
       </c>
     </row>
     <row r="50" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B50" s="6" t="s">
+      <c r="B50" s="4" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="51" spans="2:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="B51" s="7" t="s">
+      <c r="B51" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C51" s="7" cm="1" vm="2">
+      <c r="C51" s="5" cm="1" vm="2">
         <f t="array" ref="C51">_xlfn._xlws.PY(0,1)</f>
         <v>0</v>
       </c>
@@ -2090,16 +2090,16 @@
       <c r="C53"/>
     </row>
     <row r="54" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B54" s="6" t="s">
+      <c r="B54" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C54" s="6"/>
+      <c r="C54" s="4"/>
     </row>
     <row r="55" spans="2:3" ht="120" x14ac:dyDescent="0.25">
-      <c r="B55" s="7" t="s">
+      <c r="B55" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C55" s="7" t="e" cm="1" vm="3">
+      <c r="C55" s="5" t="e" cm="1" vm="3">
         <f t="array" ref="C55">_xlfn._xlws.PY(1,1,WordcloudStopwordsTable[[#All],[Stop words]])</f>
         <v>#VALUE!</v>
       </c>
@@ -2109,10 +2109,10 @@
       <c r="C56"/>
     </row>
     <row r="57" spans="2:3" ht="135" x14ac:dyDescent="0.25">
-      <c r="B57" s="7" t="s">
+      <c r="B57" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C57" s="7" t="e" cm="1" vm="4">
+      <c r="C57" s="5" t="e" cm="1" vm="4">
         <f t="array" ref="C57">_xlfn._xlws.PY(2,1,WordcloudCommentsTable[#All])</f>
         <v>#VALUE!</v>
       </c>
@@ -2122,16 +2122,16 @@
       <c r="C58"/>
     </row>
     <row r="59" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="6" t="s">
+      <c r="B59" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="C59" s="6"/>
+      <c r="C59" s="4"/>
     </row>
     <row r="60" spans="2:3" ht="165" x14ac:dyDescent="0.25">
-      <c r="B60" s="7" t="s">
+      <c r="B60" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C60" s="7" t="e" cm="1" vm="5">
+      <c r="C60" s="5" t="e" cm="1" vm="5">
         <f t="array" ref="C60">_xlfn._xlws.PY(3,1)</f>
         <v>#VALUE!</v>
       </c>
@@ -2141,16 +2141,16 @@
       <c r="C61"/>
     </row>
     <row r="62" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B62" s="6" t="s">
+      <c r="B62" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C62" s="6"/>
-    </row>
-    <row r="63" spans="2:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="B63" s="7" t="s">
+      <c r="C62" s="4"/>
+    </row>
+    <row r="63" spans="2:3" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="B63" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C63" s="7" t="str" cm="1" vm="6">
+      <c r="C63" s="5" t="str" cm="1" vm="6">
         <f t="array" ref="C63">_xlfn._xlws.PY(4,1)</f>
         <v>Absolutely love this coffee shop! The espresso is rich and smooth, and the ambiance is perfect for working or relaxing. The baristas are incredibly friendly and knowledgeable—they make the best flat white in town! A cozy little gem with fantastic pastries and the most aromatic coffee I've had in ages. I keep coming back for their pour-over coffee—so well-balanced and flavorful! The decor is stylish, the seats are comfortable, and the music is just the right volume. Their homemade syrups add such a unique twist to classic drinks—try the vanilla bean latte! Fast service, great coffee, and an overall welcoming vibe. A must-visit! A bit pricey, but the quality of the coffee and the experience make it worth every penny. This place is my go-to for a quiet morning coffee before work. Always consistent and delicious! Tried their cold brew, and it was phenomenal—strong, smooth, and not bitter at all. Great selection of alternative milks, making it super vegan-friendly. The latte art here is next-level. Almost too pretty to drink… but I do, and it’s always perfect! The staff remembers my name and order—feels like my second home! Their seasonal specials are always creative and delicious—I wish they kept them year-round! Love the community feel here. Great place to meet friends or even network with locals. I appreciate that they use ethically sourced beans. Makes me enjoy my coffee even more! Super fast WiFi, plenty of plugs, and comfortable seating make it a great spot to work remotely. The outdoor seating is a huge plus, especially on a sunny day! The croissants are buttery and flaky—pairs perfectly with their cappuccino! Sometimes the wait can be long, but it's worth it for the quality and care they put into each drink. Such a warm and inviting space! The rustic design and soft lighting make it so cozy. Their mocha is the perfect blend of rich chocolate and bold espresso—my new favorite treat! Friendly service, delicious drinks, and a laid-back atmosphere. What more could you ask for? Tried their espresso flight—such a fun way to experience different roasts and flavors! A true coffee lover's paradise. Every sip is pure perfection!</v>
       </c>
@@ -2160,16 +2160,16 @@
       <c r="C64"/>
     </row>
     <row r="65" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B65" s="6" t="s">
+      <c r="B65" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C65" s="6"/>
+      <c r="C65" s="4"/>
     </row>
     <row r="66" spans="2:3" ht="225" x14ac:dyDescent="0.25">
-      <c r="B66" s="7" t="s">
+      <c r="B66" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C66" s="7" t="e" cm="1" vm="7">
+      <c r="C66" s="5" t="e" cm="1" vm="7">
         <f t="array" ref="C66">_xlfn._xlws.PY(5,1)</f>
         <v>#VALUE!</v>
       </c>
@@ -2179,16 +2179,16 @@
       <c r="C67"/>
     </row>
     <row r="68" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B68" s="6" t="s">
+      <c r="B68" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C68" s="6"/>
+      <c r="C68" s="4"/>
     </row>
     <row r="69" spans="2:3" ht="75" x14ac:dyDescent="0.25">
-      <c r="B69" s="7" t="s">
+      <c r="B69" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="C69" s="7" t="e" cm="1" vm="8">
+      <c r="C69" s="5" t="e" cm="1" vm="8">
         <f t="array" ref="C69">_xlfn._xlws.PY(6,1)</f>
         <v>#VALUE!</v>
       </c>
@@ -2230,10 +2230,10 @@
       <c r="C77"/>
     </row>
     <row r="78" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B78" s="8" t="s">
+      <c r="B78" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C78" s="8" cm="1" vm="2">
+      <c r="C78" s="6" cm="1" vm="2">
         <f t="array" ref="C78">_xlfn._xlws.PY(7,1)</f>
         <v>0</v>
       </c>
@@ -2243,10 +2243,10 @@
       <c r="C79"/>
     </row>
     <row r="80" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B80" s="9" t="s">
+      <c r="B80" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="C80" s="10" t="s">
+      <c r="C80" s="8" t="s">
         <v>56</v>
       </c>
     </row>
@@ -2255,10 +2255,10 @@
       <c r="C81"/>
     </row>
     <row r="82" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B82" s="8" t="s">
+      <c r="B82" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="C82" s="8" t="e" cm="1" vm="9">
+      <c r="C82" s="6" t="e" cm="1" vm="9">
         <f t="array" ref="C82">_xlfn._xlws.PY(8,1,shape)</f>
         <v>#VALUE!</v>
       </c>

</xml_diff>